<commit_message>
Use invoice quantity (80 pcs) for advent calendar missing unit count
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011aeT9B1G5WiYwBahBNzkLu
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_La_Boheme_Cafe_CZ26014324.xlsx
+++ b/output/HS_Code_Summary_La_Boheme_Cafe_CZ26014324.xlsx
@@ -988,7 +988,7 @@
         <v>80</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="F18" s="6" t="n"/>
       <c r="G18" s="6" t="n"/>
@@ -1026,7 +1026,7 @@
         <v>6255</v>
       </c>
       <c r="E19" s="8" t="n">
-        <v>25856</v>
+        <v>25936</v>
       </c>
       <c r="F19" s="8" t="n">
         <v>1675.356</v>
@@ -4838,7 +4838,7 @@
         <v>80</v>
       </c>
       <c r="I60" s="12" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="J60" s="12" t="n">
         <v>0</v>

</xml_diff>